<commit_message>
Despliegue a Producción 2026-06-16 09:27
</commit_message>
<xml_diff>
--- a/crm asesores/migracion Prospectos.xlsx
+++ b/crm asesores/migracion Prospectos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/CRM AMBRIZ/crm asesores/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E30A9F1-334D-5341-BC62-1FB801B32B60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF41CD9F-55F1-4541-BD03-FF256EBDFE54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -50,7 +50,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -77,6 +77,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -86,7 +93,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -104,19 +111,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="thin">
         <color rgb="FF000000"/>
@@ -285,7 +279,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -293,54 +287,49 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -570,176 +559,176 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="34" t="s">
+      <c r="B1" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="34" t="s">
+      <c r="C1" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="34" t="s">
+      <c r="D1" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="34" t="s">
+      <c r="E1" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="34" t="s">
+      <c r="F1" s="31" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="5"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="7"/>
+      <c r="A2" s="32"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
     </row>
     <row r="3" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="9"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="12"/>
+      <c r="A3" s="32"/>
+      <c r="B3" s="33"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="32"/>
     </row>
     <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="9"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="12"/>
+      <c r="A4" s="32"/>
+      <c r="B4" s="33"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="32"/>
     </row>
     <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="9"/>
-      <c r="B5" s="6"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="12"/>
+      <c r="A5" s="32"/>
+      <c r="B5" s="33"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="33"/>
+      <c r="F5" s="32"/>
     </row>
     <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="9"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="12"/>
+      <c r="A6" s="32"/>
+      <c r="B6" s="33"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
     </row>
     <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="9"/>
-      <c r="B7" s="15"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="12"/>
+      <c r="A7" s="32"/>
+      <c r="B7" s="33"/>
+      <c r="C7" s="32"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="33"/>
+      <c r="F7" s="32"/>
     </row>
     <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="9"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="12"/>
+      <c r="A8" s="7"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="10"/>
     </row>
     <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="9"/>
-      <c r="B9" s="15"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="12"/>
+      <c r="A9" s="7"/>
+      <c r="B9" s="12"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="10"/>
     </row>
     <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="9"/>
-      <c r="B10" s="18"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="12"/>
+      <c r="A10" s="7"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="10"/>
     </row>
     <row r="11" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="9"/>
-      <c r="B11" s="18"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="12"/>
+      <c r="A11" s="7"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="10"/>
     </row>
     <row r="12" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="9"/>
-      <c r="B12" s="18"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="12"/>
+      <c r="A12" s="7"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="10"/>
     </row>
     <row r="13" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="9"/>
-      <c r="B13" s="18"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="12"/>
+      <c r="A13" s="7"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="10"/>
     </row>
     <row r="14" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="9"/>
-      <c r="B14" s="20"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="12"/>
+      <c r="A14" s="7"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="10"/>
     </row>
     <row r="15" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="9"/>
-      <c r="B15" s="20"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="12"/>
+      <c r="A15" s="7"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="10"/>
     </row>
     <row r="16" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" s="9"/>
-      <c r="B16" s="18"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="12"/>
+      <c r="A16" s="7"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="10"/>
     </row>
     <row r="17" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="9"/>
-      <c r="B17" s="18"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="12"/>
+      <c r="A17" s="7"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="10"/>
     </row>
     <row r="18" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A18" s="9"/>
-      <c r="B18" s="18"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="12"/>
+      <c r="A18" s="7"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="10"/>
     </row>
     <row r="19" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A19" s="9"/>
-      <c r="B19" s="18"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="21"/>
+      <c r="A19" s="7"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="18"/>
     </row>
     <row r="20" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A20" s="9"/>
-      <c r="B20" s="20"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="12"/>
+      <c r="A20" s="7"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="10"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
@@ -754,12 +743,12 @@
       <c r="R20" s="4"/>
     </row>
     <row r="21" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A21" s="9"/>
-      <c r="B21" s="20"/>
-      <c r="C21" s="19"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="23"/>
+      <c r="A21" s="7"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="20"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
@@ -774,580 +763,580 @@
       <c r="R21" s="4"/>
     </row>
     <row r="22" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" s="9"/>
-      <c r="B22" s="20"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="12"/>
+      <c r="A22" s="7"/>
+      <c r="B22" s="17"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="10"/>
     </row>
     <row r="23" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A23" s="9"/>
-      <c r="B23" s="20"/>
-      <c r="C23" s="19"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="12"/>
+      <c r="A23" s="7"/>
+      <c r="B23" s="17"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="10"/>
     </row>
     <row r="24" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A24" s="9"/>
-      <c r="B24" s="20"/>
-      <c r="C24" s="19"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="12"/>
+      <c r="A24" s="7"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="16"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="10"/>
     </row>
     <row r="25" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A25" s="9"/>
-      <c r="B25" s="20"/>
-      <c r="C25" s="19"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="12"/>
+      <c r="A25" s="7"/>
+      <c r="B25" s="17"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="10"/>
     </row>
     <row r="26" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A26" s="9"/>
-      <c r="B26" s="20"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="12"/>
+      <c r="A26" s="7"/>
+      <c r="B26" s="17"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="10"/>
     </row>
     <row r="27" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A27" s="9"/>
-      <c r="B27" s="20"/>
-      <c r="C27" s="19"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="11"/>
-      <c r="F27" s="24"/>
+      <c r="A27" s="7"/>
+      <c r="B27" s="17"/>
+      <c r="C27" s="16"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="21"/>
     </row>
     <row r="28" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A28" s="9"/>
-      <c r="B28" s="20"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="12"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="24"/>
+      <c r="A28" s="7"/>
+      <c r="B28" s="17"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="21"/>
     </row>
     <row r="29" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A29" s="9"/>
-      <c r="B29" s="20"/>
-      <c r="C29" s="19"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="11"/>
-      <c r="F29" s="12"/>
+      <c r="A29" s="7"/>
+      <c r="B29" s="17"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="9"/>
+      <c r="F29" s="10"/>
     </row>
     <row r="30" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A30" s="9"/>
-      <c r="B30" s="20"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="12"/>
+      <c r="A30" s="7"/>
+      <c r="B30" s="17"/>
+      <c r="C30" s="16"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="10"/>
     </row>
     <row r="31" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A31" s="9"/>
-      <c r="B31" s="20"/>
-      <c r="C31" s="19"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="11"/>
-      <c r="F31" s="12"/>
+      <c r="A31" s="7"/>
+      <c r="B31" s="17"/>
+      <c r="C31" s="16"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="9"/>
+      <c r="F31" s="10"/>
     </row>
     <row r="32" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A32" s="9"/>
-      <c r="B32" s="20"/>
-      <c r="C32" s="19"/>
+      <c r="A32" s="7"/>
+      <c r="B32" s="17"/>
+      <c r="C32" s="16"/>
       <c r="D32" s="4"/>
-      <c r="E32" s="11"/>
-      <c r="F32" s="12"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="10"/>
     </row>
     <row r="33" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A33" s="9"/>
-      <c r="B33" s="20"/>
-      <c r="C33" s="25"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="26"/>
-      <c r="F33" s="12"/>
+      <c r="A33" s="7"/>
+      <c r="B33" s="17"/>
+      <c r="C33" s="22"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="23"/>
+      <c r="F33" s="10"/>
     </row>
     <row r="34" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A34" s="9"/>
-      <c r="B34" s="20"/>
-      <c r="C34" s="25"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="26"/>
-      <c r="F34" s="12"/>
+      <c r="A34" s="7"/>
+      <c r="B34" s="17"/>
+      <c r="C34" s="22"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="23"/>
+      <c r="F34" s="10"/>
     </row>
     <row r="35" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A35" s="9"/>
-      <c r="B35" s="20"/>
-      <c r="C35" s="19"/>
-      <c r="D35" s="16"/>
-      <c r="E35" s="11"/>
-      <c r="F35" s="12"/>
+      <c r="A35" s="7"/>
+      <c r="B35" s="17"/>
+      <c r="C35" s="16"/>
+      <c r="D35" s="13"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="10"/>
     </row>
     <row r="36" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A36" s="9"/>
-      <c r="B36" s="20"/>
-      <c r="C36" s="19"/>
-      <c r="D36" s="16"/>
-      <c r="E36" s="11"/>
-      <c r="F36" s="12"/>
+      <c r="A36" s="7"/>
+      <c r="B36" s="17"/>
+      <c r="C36" s="16"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="10"/>
     </row>
     <row r="37" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A37" s="9"/>
-      <c r="B37" s="20"/>
-      <c r="C37" s="19"/>
-      <c r="D37" s="16"/>
-      <c r="E37" s="11"/>
-      <c r="F37" s="12"/>
+      <c r="A37" s="7"/>
+      <c r="B37" s="17"/>
+      <c r="C37" s="16"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="10"/>
     </row>
     <row r="38" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A38" s="9"/>
-      <c r="B38" s="20"/>
-      <c r="C38" s="19"/>
-      <c r="D38" s="16"/>
-      <c r="E38" s="11"/>
-      <c r="F38" s="12"/>
+      <c r="A38" s="7"/>
+      <c r="B38" s="17"/>
+      <c r="C38" s="16"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="10"/>
     </row>
     <row r="39" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A39" s="9"/>
-      <c r="B39" s="20"/>
-      <c r="C39" s="19"/>
-      <c r="D39" s="16"/>
-      <c r="E39" s="11"/>
-      <c r="F39" s="12"/>
+      <c r="A39" s="7"/>
+      <c r="B39" s="17"/>
+      <c r="C39" s="16"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="10"/>
     </row>
     <row r="40" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A40" s="9"/>
-      <c r="B40" s="20"/>
-      <c r="C40" s="19"/>
-      <c r="D40" s="16"/>
-      <c r="E40" s="11"/>
-      <c r="F40" s="12"/>
+      <c r="A40" s="7"/>
+      <c r="B40" s="17"/>
+      <c r="C40" s="16"/>
+      <c r="D40" s="13"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="10"/>
     </row>
     <row r="41" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A41" s="9"/>
-      <c r="B41" s="20"/>
-      <c r="C41" s="19"/>
-      <c r="D41" s="16"/>
-      <c r="E41" s="11"/>
-      <c r="F41" s="12"/>
+      <c r="A41" s="7"/>
+      <c r="B41" s="17"/>
+      <c r="C41" s="16"/>
+      <c r="D41" s="13"/>
+      <c r="E41" s="9"/>
+      <c r="F41" s="10"/>
     </row>
     <row r="42" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A42" s="9"/>
-      <c r="B42" s="20"/>
-      <c r="C42" s="19"/>
-      <c r="D42" s="16"/>
-      <c r="E42" s="11"/>
-      <c r="F42" s="12"/>
+      <c r="A42" s="7"/>
+      <c r="B42" s="17"/>
+      <c r="C42" s="16"/>
+      <c r="D42" s="13"/>
+      <c r="E42" s="9"/>
+      <c r="F42" s="10"/>
     </row>
     <row r="43" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A43" s="9"/>
-      <c r="B43" s="20"/>
-      <c r="C43" s="19"/>
-      <c r="D43" s="16"/>
-      <c r="E43" s="11"/>
-      <c r="F43" s="12"/>
+      <c r="A43" s="7"/>
+      <c r="B43" s="17"/>
+      <c r="C43" s="16"/>
+      <c r="D43" s="13"/>
+      <c r="E43" s="9"/>
+      <c r="F43" s="10"/>
     </row>
     <row r="44" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A44" s="9"/>
-      <c r="B44" s="20"/>
-      <c r="C44" s="19"/>
-      <c r="D44" s="16"/>
-      <c r="E44" s="11"/>
-      <c r="F44" s="12"/>
+      <c r="A44" s="7"/>
+      <c r="B44" s="17"/>
+      <c r="C44" s="16"/>
+      <c r="D44" s="13"/>
+      <c r="E44" s="9"/>
+      <c r="F44" s="10"/>
     </row>
     <row r="45" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A45" s="9"/>
-      <c r="B45" s="20"/>
-      <c r="C45" s="19"/>
-      <c r="D45" s="16"/>
-      <c r="E45" s="11"/>
-      <c r="F45" s="12"/>
+      <c r="A45" s="7"/>
+      <c r="B45" s="17"/>
+      <c r="C45" s="16"/>
+      <c r="D45" s="13"/>
+      <c r="E45" s="9"/>
+      <c r="F45" s="10"/>
     </row>
     <row r="46" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A46" s="9"/>
-      <c r="B46" s="20"/>
-      <c r="C46" s="19"/>
-      <c r="D46" s="16"/>
-      <c r="E46" s="11"/>
-      <c r="F46" s="12"/>
+      <c r="A46" s="7"/>
+      <c r="B46" s="17"/>
+      <c r="C46" s="16"/>
+      <c r="D46" s="13"/>
+      <c r="E46" s="9"/>
+      <c r="F46" s="10"/>
     </row>
     <row r="47" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A47" s="9"/>
-      <c r="B47" s="20"/>
-      <c r="C47" s="19"/>
-      <c r="D47" s="16"/>
-      <c r="E47" s="11"/>
-      <c r="F47" s="24"/>
+      <c r="A47" s="7"/>
+      <c r="B47" s="17"/>
+      <c r="C47" s="16"/>
+      <c r="D47" s="13"/>
+      <c r="E47" s="9"/>
+      <c r="F47" s="21"/>
     </row>
     <row r="48" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A48" s="9"/>
-      <c r="B48" s="20"/>
-      <c r="C48" s="19"/>
-      <c r="D48" s="16"/>
-      <c r="E48" s="11"/>
-      <c r="F48" s="12"/>
+      <c r="A48" s="7"/>
+      <c r="B48" s="17"/>
+      <c r="C48" s="16"/>
+      <c r="D48" s="13"/>
+      <c r="E48" s="9"/>
+      <c r="F48" s="10"/>
     </row>
     <row r="49" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A49" s="9"/>
-      <c r="B49" s="20"/>
-      <c r="C49" s="19"/>
-      <c r="D49" s="16"/>
-      <c r="E49" s="11"/>
-      <c r="F49" s="12"/>
+      <c r="A49" s="7"/>
+      <c r="B49" s="17"/>
+      <c r="C49" s="16"/>
+      <c r="D49" s="13"/>
+      <c r="E49" s="9"/>
+      <c r="F49" s="10"/>
     </row>
     <row r="50" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A50" s="9"/>
-      <c r="B50" s="20"/>
-      <c r="C50" s="19"/>
-      <c r="D50" s="16"/>
-      <c r="E50" s="11"/>
-      <c r="F50" s="12"/>
+      <c r="A50" s="7"/>
+      <c r="B50" s="17"/>
+      <c r="C50" s="16"/>
+      <c r="D50" s="13"/>
+      <c r="E50" s="9"/>
+      <c r="F50" s="10"/>
     </row>
     <row r="51" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A51" s="9"/>
-      <c r="B51" s="20"/>
-      <c r="C51" s="19"/>
-      <c r="D51" s="16"/>
-      <c r="E51" s="11"/>
-      <c r="F51" s="12"/>
+      <c r="A51" s="7"/>
+      <c r="B51" s="17"/>
+      <c r="C51" s="16"/>
+      <c r="D51" s="13"/>
+      <c r="E51" s="9"/>
+      <c r="F51" s="10"/>
     </row>
     <row r="52" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A52" s="9"/>
-      <c r="B52" s="20"/>
-      <c r="C52" s="19"/>
-      <c r="D52" s="16"/>
-      <c r="E52" s="11"/>
-      <c r="F52" s="12"/>
+      <c r="A52" s="7"/>
+      <c r="B52" s="17"/>
+      <c r="C52" s="16"/>
+      <c r="D52" s="13"/>
+      <c r="E52" s="9"/>
+      <c r="F52" s="10"/>
     </row>
     <row r="53" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A53" s="9"/>
-      <c r="B53" s="20"/>
-      <c r="C53" s="19"/>
-      <c r="D53" s="16"/>
-      <c r="E53" s="11"/>
-      <c r="F53" s="12"/>
+      <c r="A53" s="7"/>
+      <c r="B53" s="17"/>
+      <c r="C53" s="16"/>
+      <c r="D53" s="13"/>
+      <c r="E53" s="9"/>
+      <c r="F53" s="10"/>
     </row>
     <row r="54" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A54" s="9"/>
-      <c r="B54" s="20"/>
-      <c r="C54" s="19"/>
-      <c r="D54" s="16"/>
-      <c r="E54" s="11"/>
-      <c r="F54" s="12"/>
+      <c r="A54" s="7"/>
+      <c r="B54" s="17"/>
+      <c r="C54" s="16"/>
+      <c r="D54" s="13"/>
+      <c r="E54" s="9"/>
+      <c r="F54" s="10"/>
     </row>
     <row r="55" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A55" s="9"/>
-      <c r="B55" s="20"/>
-      <c r="C55" s="19"/>
-      <c r="D55" s="16"/>
-      <c r="E55" s="11"/>
-      <c r="F55" s="12"/>
+      <c r="A55" s="7"/>
+      <c r="B55" s="17"/>
+      <c r="C55" s="16"/>
+      <c r="D55" s="13"/>
+      <c r="E55" s="9"/>
+      <c r="F55" s="10"/>
     </row>
     <row r="56" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A56" s="9"/>
-      <c r="B56" s="20"/>
-      <c r="C56" s="19"/>
-      <c r="D56" s="16"/>
-      <c r="E56" s="11"/>
-      <c r="F56" s="12"/>
+      <c r="A56" s="7"/>
+      <c r="B56" s="17"/>
+      <c r="C56" s="16"/>
+      <c r="D56" s="13"/>
+      <c r="E56" s="9"/>
+      <c r="F56" s="10"/>
     </row>
     <row r="57" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A57" s="9"/>
-      <c r="B57" s="20"/>
-      <c r="C57" s="19"/>
-      <c r="D57" s="16"/>
-      <c r="E57" s="11"/>
-      <c r="F57" s="12"/>
+      <c r="A57" s="7"/>
+      <c r="B57" s="17"/>
+      <c r="C57" s="16"/>
+      <c r="D57" s="13"/>
+      <c r="E57" s="9"/>
+      <c r="F57" s="10"/>
     </row>
     <row r="58" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A58" s="9"/>
-      <c r="B58" s="20"/>
-      <c r="C58" s="19"/>
-      <c r="D58" s="16"/>
-      <c r="E58" s="11"/>
-      <c r="F58" s="12"/>
+      <c r="A58" s="7"/>
+      <c r="B58" s="17"/>
+      <c r="C58" s="16"/>
+      <c r="D58" s="13"/>
+      <c r="E58" s="9"/>
+      <c r="F58" s="10"/>
     </row>
     <row r="59" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A59" s="9"/>
-      <c r="B59" s="20"/>
-      <c r="C59" s="19"/>
-      <c r="D59" s="16"/>
-      <c r="E59" s="11"/>
-      <c r="F59" s="12"/>
+      <c r="A59" s="7"/>
+      <c r="B59" s="17"/>
+      <c r="C59" s="16"/>
+      <c r="D59" s="13"/>
+      <c r="E59" s="9"/>
+      <c r="F59" s="10"/>
     </row>
     <row r="60" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A60" s="9"/>
-      <c r="B60" s="20"/>
-      <c r="C60" s="19"/>
-      <c r="D60" s="16"/>
-      <c r="E60" s="11"/>
-      <c r="F60" s="12"/>
+      <c r="A60" s="7"/>
+      <c r="B60" s="17"/>
+      <c r="C60" s="16"/>
+      <c r="D60" s="13"/>
+      <c r="E60" s="9"/>
+      <c r="F60" s="10"/>
     </row>
     <row r="61" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A61" s="9"/>
-      <c r="B61" s="20"/>
-      <c r="C61" s="19"/>
-      <c r="D61" s="16"/>
-      <c r="E61" s="11"/>
-      <c r="F61" s="12"/>
+      <c r="A61" s="7"/>
+      <c r="B61" s="17"/>
+      <c r="C61" s="16"/>
+      <c r="D61" s="13"/>
+      <c r="E61" s="9"/>
+      <c r="F61" s="10"/>
     </row>
     <row r="62" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A62" s="9"/>
-      <c r="B62" s="20"/>
-      <c r="C62" s="19"/>
-      <c r="D62" s="16"/>
-      <c r="E62" s="11"/>
-      <c r="F62" s="12"/>
+      <c r="A62" s="7"/>
+      <c r="B62" s="17"/>
+      <c r="C62" s="16"/>
+      <c r="D62" s="13"/>
+      <c r="E62" s="9"/>
+      <c r="F62" s="10"/>
     </row>
     <row r="63" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A63" s="9"/>
-      <c r="B63" s="20"/>
-      <c r="C63" s="19"/>
-      <c r="D63" s="16"/>
-      <c r="E63" s="11"/>
-      <c r="F63" s="12"/>
+      <c r="A63" s="7"/>
+      <c r="B63" s="17"/>
+      <c r="C63" s="16"/>
+      <c r="D63" s="13"/>
+      <c r="E63" s="9"/>
+      <c r="F63" s="10"/>
     </row>
     <row r="64" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A64" s="27"/>
-      <c r="B64" s="28"/>
-      <c r="C64" s="29"/>
-      <c r="D64" s="30"/>
-      <c r="E64" s="31"/>
-      <c r="F64" s="21"/>
+      <c r="A64" s="24"/>
+      <c r="B64" s="25"/>
+      <c r="C64" s="26"/>
+      <c r="D64" s="27"/>
+      <c r="E64" s="28"/>
+      <c r="F64" s="18"/>
     </row>
     <row r="65" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A65" s="12"/>
-      <c r="B65" s="13"/>
-      <c r="C65" s="12"/>
-      <c r="D65" s="30"/>
-      <c r="E65" s="11"/>
-      <c r="F65" s="12"/>
+      <c r="A65" s="10"/>
+      <c r="B65" s="11"/>
+      <c r="C65" s="10"/>
+      <c r="D65" s="27"/>
+      <c r="E65" s="9"/>
+      <c r="F65" s="10"/>
     </row>
     <row r="66" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A66" s="12"/>
-      <c r="B66" s="13"/>
-      <c r="C66" s="12"/>
-      <c r="D66" s="30"/>
-      <c r="E66" s="11"/>
-      <c r="F66" s="16"/>
+      <c r="A66" s="10"/>
+      <c r="B66" s="11"/>
+      <c r="C66" s="10"/>
+      <c r="D66" s="27"/>
+      <c r="E66" s="9"/>
+      <c r="F66" s="13"/>
     </row>
     <row r="67" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A67" s="12"/>
-      <c r="B67" s="13"/>
-      <c r="C67" s="12"/>
-      <c r="D67" s="30"/>
-      <c r="E67" s="11"/>
-      <c r="F67" s="24"/>
+      <c r="A67" s="10"/>
+      <c r="B67" s="11"/>
+      <c r="C67" s="10"/>
+      <c r="D67" s="27"/>
+      <c r="E67" s="9"/>
+      <c r="F67" s="21"/>
     </row>
     <row r="68" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A68" s="12"/>
-      <c r="B68" s="13"/>
-      <c r="C68" s="12"/>
-      <c r="D68" s="30"/>
-      <c r="E68" s="11"/>
-      <c r="F68" s="16"/>
+      <c r="A68" s="10"/>
+      <c r="B68" s="11"/>
+      <c r="C68" s="10"/>
+      <c r="D68" s="27"/>
+      <c r="E68" s="9"/>
+      <c r="F68" s="13"/>
     </row>
     <row r="69" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A69" s="12"/>
-      <c r="B69" s="13"/>
-      <c r="C69" s="12"/>
-      <c r="D69" s="30"/>
-      <c r="E69" s="11"/>
-      <c r="F69" s="16"/>
+      <c r="A69" s="10"/>
+      <c r="B69" s="11"/>
+      <c r="C69" s="10"/>
+      <c r="D69" s="27"/>
+      <c r="E69" s="9"/>
+      <c r="F69" s="13"/>
     </row>
     <row r="70" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A70" s="12"/>
-      <c r="B70" s="13"/>
-      <c r="C70" s="12"/>
-      <c r="D70" s="30"/>
-      <c r="E70" s="11"/>
-      <c r="F70" s="16"/>
+      <c r="A70" s="10"/>
+      <c r="B70" s="11"/>
+      <c r="C70" s="10"/>
+      <c r="D70" s="27"/>
+      <c r="E70" s="9"/>
+      <c r="F70" s="13"/>
     </row>
     <row r="71" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A71" s="12"/>
-      <c r="B71" s="13"/>
-      <c r="C71" s="12"/>
-      <c r="D71" s="16"/>
-      <c r="E71" s="11"/>
-      <c r="F71" s="16"/>
+      <c r="A71" s="10"/>
+      <c r="B71" s="11"/>
+      <c r="C71" s="10"/>
+      <c r="D71" s="13"/>
+      <c r="E71" s="9"/>
+      <c r="F71" s="13"/>
     </row>
     <row r="72" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A72" s="32"/>
-      <c r="B72" s="33"/>
-      <c r="C72" s="21"/>
-      <c r="D72" s="30"/>
-      <c r="E72" s="31"/>
-      <c r="F72" s="30"/>
+      <c r="A72" s="29"/>
+      <c r="B72" s="30"/>
+      <c r="C72" s="18"/>
+      <c r="D72" s="27"/>
+      <c r="E72" s="28"/>
+      <c r="F72" s="27"/>
     </row>
     <row r="73" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A73" s="12"/>
-      <c r="B73" s="13"/>
-      <c r="C73" s="12"/>
-      <c r="D73" s="16"/>
-      <c r="E73" s="11"/>
-      <c r="F73" s="24"/>
+      <c r="A73" s="10"/>
+      <c r="B73" s="11"/>
+      <c r="C73" s="10"/>
+      <c r="D73" s="13"/>
+      <c r="E73" s="9"/>
+      <c r="F73" s="21"/>
     </row>
     <row r="74" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A74" s="12"/>
-      <c r="B74" s="13"/>
-      <c r="C74" s="12"/>
-      <c r="D74" s="16"/>
-      <c r="E74" s="11"/>
-      <c r="F74" s="16"/>
+      <c r="A74" s="10"/>
+      <c r="B74" s="11"/>
+      <c r="C74" s="10"/>
+      <c r="D74" s="13"/>
+      <c r="E74" s="9"/>
+      <c r="F74" s="13"/>
     </row>
     <row r="75" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A75" s="12"/>
-      <c r="B75" s="13"/>
-      <c r="C75" s="12"/>
-      <c r="D75" s="16"/>
-      <c r="E75" s="11"/>
-      <c r="F75" s="16"/>
+      <c r="A75" s="10"/>
+      <c r="B75" s="11"/>
+      <c r="C75" s="10"/>
+      <c r="D75" s="13"/>
+      <c r="E75" s="9"/>
+      <c r="F75" s="13"/>
     </row>
     <row r="76" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A76" s="12"/>
-      <c r="B76" s="13"/>
-      <c r="C76" s="12"/>
-      <c r="D76" s="16"/>
-      <c r="E76" s="11"/>
-      <c r="F76" s="16"/>
+      <c r="A76" s="10"/>
+      <c r="B76" s="11"/>
+      <c r="C76" s="10"/>
+      <c r="D76" s="13"/>
+      <c r="E76" s="9"/>
+      <c r="F76" s="13"/>
     </row>
     <row r="77" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A77" s="12"/>
-      <c r="B77" s="13"/>
-      <c r="C77" s="12"/>
-      <c r="D77" s="16"/>
-      <c r="E77" s="11"/>
-      <c r="F77" s="16"/>
+      <c r="A77" s="10"/>
+      <c r="B77" s="11"/>
+      <c r="C77" s="10"/>
+      <c r="D77" s="13"/>
+      <c r="E77" s="9"/>
+      <c r="F77" s="13"/>
     </row>
     <row r="78" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A78" s="12"/>
-      <c r="B78" s="13"/>
-      <c r="C78" s="12"/>
-      <c r="D78" s="16"/>
-      <c r="E78" s="11"/>
-      <c r="F78" s="16"/>
+      <c r="A78" s="10"/>
+      <c r="B78" s="11"/>
+      <c r="C78" s="10"/>
+      <c r="D78" s="13"/>
+      <c r="E78" s="9"/>
+      <c r="F78" s="13"/>
     </row>
     <row r="79" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A79" s="12"/>
-      <c r="B79" s="13"/>
-      <c r="C79" s="12"/>
-      <c r="D79" s="16"/>
-      <c r="E79" s="11"/>
-      <c r="F79" s="16"/>
+      <c r="A79" s="10"/>
+      <c r="B79" s="11"/>
+      <c r="C79" s="10"/>
+      <c r="D79" s="13"/>
+      <c r="E79" s="9"/>
+      <c r="F79" s="13"/>
     </row>
     <row r="80" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A80" s="12"/>
-      <c r="B80" s="13"/>
-      <c r="C80" s="12"/>
-      <c r="D80" s="16"/>
-      <c r="E80" s="11"/>
-      <c r="F80" s="16"/>
+      <c r="A80" s="10"/>
+      <c r="B80" s="11"/>
+      <c r="C80" s="10"/>
+      <c r="D80" s="13"/>
+      <c r="E80" s="9"/>
+      <c r="F80" s="13"/>
     </row>
     <row r="81" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A81" s="21"/>
-      <c r="B81" s="33"/>
-      <c r="C81" s="21"/>
-      <c r="D81" s="30"/>
-      <c r="E81" s="31"/>
-      <c r="F81" s="30"/>
+      <c r="A81" s="18"/>
+      <c r="B81" s="30"/>
+      <c r="C81" s="18"/>
+      <c r="D81" s="27"/>
+      <c r="E81" s="28"/>
+      <c r="F81" s="27"/>
     </row>
     <row r="82" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A82" s="12"/>
-      <c r="B82" s="13"/>
-      <c r="C82" s="12"/>
-      <c r="D82" s="16"/>
-      <c r="E82" s="11"/>
-      <c r="F82" s="16"/>
+      <c r="A82" s="10"/>
+      <c r="B82" s="11"/>
+      <c r="C82" s="10"/>
+      <c r="D82" s="13"/>
+      <c r="E82" s="9"/>
+      <c r="F82" s="13"/>
     </row>
     <row r="83" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A83" s="12"/>
-      <c r="B83" s="13"/>
-      <c r="C83" s="12"/>
-      <c r="D83" s="16"/>
-      <c r="E83" s="11"/>
-      <c r="F83" s="16"/>
+      <c r="A83" s="10"/>
+      <c r="B83" s="11"/>
+      <c r="C83" s="10"/>
+      <c r="D83" s="13"/>
+      <c r="E83" s="9"/>
+      <c r="F83" s="13"/>
     </row>
     <row r="84" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A84" s="12"/>
-      <c r="B84" s="13"/>
-      <c r="C84" s="12"/>
-      <c r="D84" s="16"/>
-      <c r="E84" s="11"/>
-      <c r="F84" s="16"/>
+      <c r="A84" s="10"/>
+      <c r="B84" s="11"/>
+      <c r="C84" s="10"/>
+      <c r="D84" s="13"/>
+      <c r="E84" s="9"/>
+      <c r="F84" s="13"/>
     </row>
     <row r="85" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A85" s="12"/>
-      <c r="B85" s="13"/>
-      <c r="C85" s="12"/>
-      <c r="D85" s="16"/>
-      <c r="E85" s="11"/>
-      <c r="F85" s="16"/>
+      <c r="A85" s="10"/>
+      <c r="B85" s="11"/>
+      <c r="C85" s="10"/>
+      <c r="D85" s="13"/>
+      <c r="E85" s="9"/>
+      <c r="F85" s="13"/>
     </row>
     <row r="86" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A86" s="12"/>
-      <c r="B86" s="13"/>
-      <c r="C86" s="12"/>
-      <c r="D86" s="16"/>
-      <c r="E86" s="11"/>
-      <c r="F86" s="16"/>
+      <c r="A86" s="10"/>
+      <c r="B86" s="11"/>
+      <c r="C86" s="10"/>
+      <c r="D86" s="13"/>
+      <c r="E86" s="9"/>
+      <c r="F86" s="13"/>
     </row>
     <row r="87" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A87" s="12"/>
-      <c r="B87" s="13"/>
-      <c r="C87" s="12"/>
-      <c r="D87" s="16"/>
-      <c r="E87" s="11"/>
-      <c r="F87" s="16"/>
+      <c r="A87" s="10"/>
+      <c r="B87" s="11"/>
+      <c r="C87" s="10"/>
+      <c r="D87" s="13"/>
+      <c r="E87" s="9"/>
+      <c r="F87" s="13"/>
     </row>
     <row r="88" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A88" s="12"/>
-      <c r="B88" s="13"/>
-      <c r="C88" s="12"/>
-      <c r="D88" s="16"/>
-      <c r="E88" s="11"/>
-      <c r="F88" s="16"/>
+      <c r="A88" s="10"/>
+      <c r="B88" s="11"/>
+      <c r="C88" s="10"/>
+      <c r="D88" s="13"/>
+      <c r="E88" s="9"/>
+      <c r="F88" s="13"/>
     </row>
     <row r="89" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A89" s="32"/>
-      <c r="B89" s="33"/>
-      <c r="C89" s="21"/>
-      <c r="D89" s="30"/>
-      <c r="E89" s="31"/>
-      <c r="F89" s="30"/>
+      <c r="A89" s="29"/>
+      <c r="B89" s="30"/>
+      <c r="C89" s="18"/>
+      <c r="D89" s="27"/>
+      <c r="E89" s="28"/>
+      <c r="F89" s="27"/>
     </row>
     <row r="90" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A90" s="12"/>
-      <c r="B90" s="13"/>
-      <c r="C90" s="12"/>
-      <c r="D90" s="16"/>
-      <c r="E90" s="11"/>
-      <c r="F90" s="16"/>
+      <c r="A90" s="10"/>
+      <c r="B90" s="11"/>
+      <c r="C90" s="10"/>
+      <c r="D90" s="13"/>
+      <c r="E90" s="9"/>
+      <c r="F90" s="13"/>
     </row>
     <row r="91" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A91" s="12"/>
-      <c r="B91" s="13"/>
-      <c r="C91" s="12"/>
-      <c r="D91" s="16"/>
-      <c r="E91" s="11"/>
-      <c r="F91" s="16"/>
+      <c r="A91" s="10"/>
+      <c r="B91" s="11"/>
+      <c r="C91" s="10"/>
+      <c r="D91" s="13"/>
+      <c r="E91" s="9"/>
+      <c r="F91" s="13"/>
     </row>
     <row r="92" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A92" s="12"/>
-      <c r="B92" s="13"/>
-      <c r="C92" s="12"/>
-      <c r="D92" s="16"/>
-      <c r="E92" s="11"/>
-      <c r="F92" s="24"/>
+      <c r="A92" s="10"/>
+      <c r="B92" s="11"/>
+      <c r="C92" s="10"/>
+      <c r="D92" s="13"/>
+      <c r="E92" s="9"/>
+      <c r="F92" s="21"/>
     </row>
     <row r="93" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A93" s="12"/>
-      <c r="B93" s="13"/>
-      <c r="C93" s="12"/>
-      <c r="D93" s="16"/>
-      <c r="E93" s="11"/>
-      <c r="F93" s="16"/>
+      <c r="A93" s="10"/>
+      <c r="B93" s="11"/>
+      <c r="C93" s="10"/>
+      <c r="D93" s="13"/>
+      <c r="E93" s="9"/>
+      <c r="F93" s="13"/>
     </row>
     <row r="94" spans="1:6" ht="13" x14ac:dyDescent="0.15">
       <c r="A94" s="1"/>

</xml_diff>